<commit_message>
Updated thesis files after revision
</commit_message>
<xml_diff>
--- a/Manuscript Variant Workbooks/Alexandrinus-to-Harley7522A_1Sam-2Kings_scribe-2_MS-spreadsheet.xlsx
+++ b/Manuscript Variant Workbooks/Alexandrinus-to-Harley7522A_1Sam-2Kings_scribe-2_MS-spreadsheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/186593bc330ab858/Cambridge PhD/Thesis/8 Corrections/Files to Upload/MS Variant Spreadsheets/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/186593bc330ab858/Cambridge PhD/Thesis/10 The Final Final Version/New and Updated Files for Upload/MS Variant Spreadsheets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="555" documentId="8_{60EDC4C5-C00E-499D-8D62-4D840DF91586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C20F2B63-BE52-48DC-B7E7-1F10F05CA442}"/>
+  <xr:revisionPtr revIDLastSave="600" documentId="8_{60EDC4C5-C00E-499D-8D62-4D840DF91586}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B62DB630-B695-4711-9028-B15E1D88019B}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{5BB4D106-A247-41F8-A104-83D51E35EC09}"/>
+    <workbookView xWindow="-19530" yWindow="-21720" windowWidth="38640" windowHeight="21120" xr2:uid="{5BB4D106-A247-41F8-A104-83D51E35EC09}"/>
   </bookViews>
   <sheets>
     <sheet name="Unfiltered Data" sheetId="4" r:id="rId1"/>
@@ -843,7 +843,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K3" authorId="1" shapeId="0" xr:uid="{A56AB05E-D2B9-47F0-BBA8-D8ACE8682F4C}">
+    <comment ref="L3" authorId="1" shapeId="0" xr:uid="{A56AB05E-D2B9-47F0-BBA8-D8ACE8682F4C}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -851,7 +851,7 @@
     The apograph reading is singular and the autograph reading is not. The singular readings method would detect this variant</t>
       </text>
     </comment>
-    <comment ref="K4" authorId="2" shapeId="0" xr:uid="{C10C6CE7-AB85-45B7-9827-5BAE13547DE4}">
+    <comment ref="L4" authorId="2" shapeId="0" xr:uid="{C10C6CE7-AB85-45B7-9827-5BAE13547DE4}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -859,7 +859,7 @@
     That is, the autograph contains a singular reading and the apograph followed it</t>
       </text>
     </comment>
-    <comment ref="K5" authorId="3" shapeId="0" xr:uid="{57358701-A47D-4BC9-A30C-4D3F9F1528F8}">
+    <comment ref="L5" authorId="3" shapeId="0" xr:uid="{57358701-A47D-4BC9-A30C-4D3F9F1528F8}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -867,7 +867,7 @@
     The apograph reading is not singular: other witnesses contain the same reading. These are real variants produced by the apograph scribe, but the singular readings method would not detect them</t>
       </text>
     </comment>
-    <comment ref="M13" authorId="4" shapeId="0" xr:uid="{DF5A39CF-53B5-40CC-9266-FAAB20A43327}">
+    <comment ref="N13" authorId="4" shapeId="0" xr:uid="{DF5A39CF-53B5-40CC-9266-FAAB20A43327}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -4516,6 +4516,15 @@
     <author>tc={E2E14910-9C21-4C37-B732-F7EBFDB74CE7}</author>
     <author>tc={4718703A-88BB-4A36-8D67-5BEEDE97AD44}</author>
     <author>tc={2A549E49-EC4D-4BCE-9D24-3587690BBE3F}</author>
+    <author>tc={02A6D890-84D1-4E3F-8AE1-24828B2D0EB7}</author>
+    <author>tc={4F295585-405A-4978-850A-33295E439C73}</author>
+    <author>tc={B6DD7816-2B78-48F4-B907-8A94AE3AACDE}</author>
+    <author>tc={74BEC885-3C8B-46BF-8438-4A7591AFFECD}</author>
+    <author>tc={D3C776AC-8270-4A3D-9B37-75231FF08A0B}</author>
+    <author>tc={FE3E8DDF-ED59-452E-AD21-E71B4BB0C0BC}</author>
+    <author>tc={3C12160F-D788-4EBD-AD28-67F56579852E}</author>
+    <author>tc={5ECFDB7C-4ACB-4B8C-9D00-20B090334AFD}</author>
+    <author>tc={920AA4EA-E225-4A97-90C2-A1AC74AD8C9B}</author>
   </authors>
   <commentList>
     <comment ref="B1" authorId="0" shapeId="0" xr:uid="{295BECCE-5B1D-49E8-AE3D-EA1B28DAAE2C}">
@@ -4921,7 +4930,7 @@
     For substitutions, the word frequency of the autograph reading</t>
       </text>
     </comment>
-    <comment ref="W1" authorId="0" shapeId="0" xr:uid="{62566C8E-F9EC-4FE7-ACB9-411C15B71B9E}">
+    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{62566C8E-F9EC-4FE7-ACB9-411C15B71B9E}">
       <text>
         <r>
           <rPr>
@@ -4945,7 +4954,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X1" authorId="0" shapeId="0" xr:uid="{9450CFD4-3FFA-406F-B0B6-1CF4BF1ED4CA}">
+    <comment ref="Y1" authorId="0" shapeId="0" xr:uid="{9450CFD4-3FFA-406F-B0B6-1CF4BF1ED4CA}">
       <text>
         <r>
           <rPr>
@@ -4969,7 +4978,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y1" authorId="0" shapeId="0" xr:uid="{1B0D2868-2CA0-4C44-860B-A1E0A81B0DE4}">
+    <comment ref="Z1" authorId="0" shapeId="0" xr:uid="{1B0D2868-2CA0-4C44-860B-A1E0A81B0DE4}">
       <text>
         <r>
           <rPr>
@@ -4993,7 +5002,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Z1" authorId="0" shapeId="0" xr:uid="{88AC2CFC-CBAE-4EF9-A6D0-DA7716CBD81F}">
+    <comment ref="AA1" authorId="0" shapeId="0" xr:uid="{88AC2CFC-CBAE-4EF9-A6D0-DA7716CBD81F}">
       <text>
         <r>
           <rPr>
@@ -5017,7 +5026,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AB1" authorId="0" shapeId="0" xr:uid="{6985E317-E20E-4353-B53B-81F418B0EBCF}">
+    <comment ref="AC1" authorId="0" shapeId="0" xr:uid="{6985E317-E20E-4353-B53B-81F418B0EBCF}">
       <text>
         <r>
           <rPr>
@@ -5042,7 +5051,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AC1" authorId="0" shapeId="0" xr:uid="{7EE8AD3B-386F-4B97-AC97-2BB6CD81053A}">
+    <comment ref="AD1" authorId="0" shapeId="0" xr:uid="{7EE8AD3B-386F-4B97-AC97-2BB6CD81053A}">
       <text>
         <r>
           <rPr>
@@ -5066,7 +5075,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD1" authorId="0" shapeId="0" xr:uid="{6B335B41-7D17-4593-99A9-24056EFE1C77}">
+    <comment ref="AE1" authorId="0" shapeId="0" xr:uid="{6B335B41-7D17-4593-99A9-24056EFE1C77}">
       <text>
         <r>
           <rPr>
@@ -5107,6 +5116,78 @@
       </text>
     </comment>
     <comment ref="D14" authorId="5" shapeId="0" xr:uid="{2A549E49-EC4D-4BCE-9D24-3587690BBE3F}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The ratio of harmonizations to disharmonizations; = harmonizations / (harmonizations + disharmonizations)</t>
+      </text>
+    </comment>
+    <comment ref="E18" authorId="6" shapeId="0" xr:uid="{02A6D890-84D1-4E3F-8AE1-24828B2D0EB7}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    ONLY those cases where influence from preceding material was possible and EXCLUDING cases where influence from following material was possible.</t>
+      </text>
+    </comment>
+    <comment ref="F18" authorId="7" shapeId="0" xr:uid="{4F295585-405A-4978-850A-33295E439C73}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    All cases where influence from preceding material was possible.</t>
+      </text>
+    </comment>
+    <comment ref="G18" authorId="8" shapeId="0" xr:uid="{B6DD7816-2B78-48F4-B907-8A94AE3AACDE}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    ONLY those cases where influence from following material was possible and EXCLUDING cases where influence from preceding material was possible.</t>
+      </text>
+    </comment>
+    <comment ref="H18" authorId="9" shapeId="0" xr:uid="{74BEC885-3C8B-46BF-8438-4A7591AFFECD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    All cases where influence from following material was possible.</t>
+      </text>
+    </comment>
+    <comment ref="I18" authorId="10" shapeId="0" xr:uid="{D3C776AC-8270-4A3D-9B37-75231FF08A0B}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Only cases where verbal parallels existed both behind and after the variant in question and the direction of change in verbal similarity was the same.</t>
+      </text>
+    </comment>
+    <comment ref="J18" authorId="11" shapeId="0" xr:uid="{FE3E8DDF-ED59-452E-AD21-E71B4BB0C0BC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    All potential cases of verbal harmonization/disharmonization, forward and backward.</t>
+      </text>
+    </comment>
+    <comment ref="D19" authorId="12" shapeId="0" xr:uid="{3C12160F-D788-4EBD-AD28-67F56579852E}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The number of variants that harmonized to parallel phrases in the near context</t>
+      </text>
+    </comment>
+    <comment ref="D20" authorId="13" shapeId="0" xr:uid="{5ECFDB7C-4ACB-4B8C-9D00-20B090334AFD}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    The number of variants that disharmonized from  parallel phrases in the near context</t>
+      </text>
+    </comment>
+    <comment ref="D21" authorId="14" shapeId="0" xr:uid="{920AA4EA-E225-4A97-90C2-A1AC74AD8C9B}">
       <text>
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
@@ -5262,7 +5343,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6080" uniqueCount="1645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6103" uniqueCount="1653">
   <si>
     <t>Verse Ref</t>
   </si>
@@ -15827,6 +15908,30 @@
   </si>
   <si>
     <t>autograph uses form as in 23:11 (και κατεκαυσαν τους ιππους ους εδωκεν βασιλευς ιουδα); apograph disharmonizes</t>
+  </si>
+  <si>
+    <t>Harmonization_Direction</t>
+  </si>
+  <si>
+    <t>Forward</t>
+  </si>
+  <si>
+    <t>Backward</t>
+  </si>
+  <si>
+    <t>Directionality</t>
+  </si>
+  <si>
+    <t>Forward (Exclusive)</t>
+  </si>
+  <si>
+    <t>Forward (Inclusive)</t>
+  </si>
+  <si>
+    <t>Backward (Exclusive)</t>
+  </si>
+  <si>
+    <t>Backward (Inclusive)</t>
   </si>
 </sst>
 </file>
@@ -18289,16 +18394,16 @@
 
 <file path=xl/threadedComments/threadedComment10.xml><?xml version="1.0" encoding="utf-8"?>
 <ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="K3" dT="2023-08-03T13:34:30.53" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{A56AB05E-D2B9-47F0-BBA8-D8ACE8682F4C}">
+  <threadedComment ref="L3" dT="2023-08-03T13:34:30.53" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{A56AB05E-D2B9-47F0-BBA8-D8ACE8682F4C}">
     <text>The apograph reading is singular and the autograph reading is not. The singular readings method would detect this variant</text>
   </threadedComment>
-  <threadedComment ref="K4" dT="2023-08-03T13:33:28.57" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{C10C6CE7-AB85-45B7-9827-5BAE13547DE4}">
+  <threadedComment ref="L4" dT="2023-08-03T13:33:28.57" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{C10C6CE7-AB85-45B7-9827-5BAE13547DE4}">
     <text>That is, the autograph contains a singular reading and the apograph followed it</text>
   </threadedComment>
-  <threadedComment ref="K5" dT="2023-08-03T13:35:10.13" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{57358701-A47D-4BC9-A30C-4D3F9F1528F8}">
+  <threadedComment ref="L5" dT="2023-08-03T13:35:10.13" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{57358701-A47D-4BC9-A30C-4D3F9F1528F8}">
     <text>The apograph reading is not singular: other witnesses contain the same reading. These are real variants produced by the apograph scribe, but the singular readings method would not detect them</text>
   </threadedComment>
-  <threadedComment ref="M13" dT="2023-08-14T14:21:11.11" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{DF5A39CF-53B5-40CC-9266-FAAB20A43327}">
+  <threadedComment ref="N13" dT="2023-08-14T14:21:11.11" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{DF5A39CF-53B5-40CC-9266-FAAB20A43327}">
     <text>For words which have multiple common forms not impacting their inflection (e.g., ουκ-ουχ-ου, επι-επ-εφ)</text>
   </threadedComment>
 </ThreadedComments>
@@ -18616,6 +18721,33 @@
   <threadedComment ref="D14" dT="2024-01-24T17:16:15.06" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{2A549E49-EC4D-4BCE-9D24-3587690BBE3F}">
     <text>The ratio of harmonizations to disharmonizations; = harmonizations / (harmonizations + disharmonizations)</text>
   </threadedComment>
+  <threadedComment ref="E18" dT="2026-03-27T21:09:00.40" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{02A6D890-84D1-4E3F-8AE1-24828B2D0EB7}">
+    <text>ONLY those cases where influence from preceding material was possible and EXCLUDING cases where influence from following material was possible.</text>
+  </threadedComment>
+  <threadedComment ref="F18" dT="2026-03-26T18:54:36.97" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{4F295585-405A-4978-850A-33295E439C73}">
+    <text>All cases where influence from preceding material was possible.</text>
+  </threadedComment>
+  <threadedComment ref="G18" dT="2026-03-27T21:09:12.56" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{B6DD7816-2B78-48F4-B907-8A94AE3AACDE}">
+    <text>ONLY those cases where influence from following material was possible and EXCLUDING cases where influence from preceding material was possible.</text>
+  </threadedComment>
+  <threadedComment ref="H18" dT="2026-03-26T18:55:05.59" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{74BEC885-3C8B-46BF-8438-4A7591AFFECD}">
+    <text>All cases where influence from following material was possible.</text>
+  </threadedComment>
+  <threadedComment ref="I18" dT="2026-03-26T18:56:11.72" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{D3C776AC-8270-4A3D-9B37-75231FF08A0B}">
+    <text>Only cases where verbal parallels existed both behind and after the variant in question and the direction of change in verbal similarity was the same.</text>
+  </threadedComment>
+  <threadedComment ref="J18" dT="2026-03-26T18:56:36.44" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{FE3E8DDF-ED59-452E-AD21-E71B4BB0C0BC}">
+    <text>All potential cases of verbal harmonization/disharmonization, forward and backward.</text>
+  </threadedComment>
+  <threadedComment ref="D19" dT="2024-01-24T17:15:11.25" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{3C12160F-D788-4EBD-AD28-67F56579852E}">
+    <text>The number of variants that harmonized to parallel phrases in the near context</text>
+  </threadedComment>
+  <threadedComment ref="D20" dT="2024-01-24T17:15:35.01" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{5ECFDB7C-4ACB-4B8C-9D00-20B090334AFD}">
+    <text>The number of variants that disharmonized from  parallel phrases in the near context</text>
+  </threadedComment>
+  <threadedComment ref="D21" dT="2024-01-24T17:16:15.06" personId="{F418FEAB-B6F1-4619-B287-21956836AF69}" id="{920AA4EA-E225-4A97-90C2-A1AC74AD8C9B}">
+    <text>The ratio of harmonizations to disharmonizations; = harmonizations / (harmonizations + disharmonizations)</text>
+  </threadedComment>
 </ThreadedComments>
 </file>
 
@@ -18655,7 +18787,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36879D5B-C28E-48E4-939D-46B2362760F6}">
-  <dimension ref="A1:AF597"/>
+  <dimension ref="A1:AF600"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
     <col min="1" max="1" width="10.81640625" customWidth="1"/>
@@ -28484,7 +28616,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="320" spans="1:31" ht="29">
+    <row r="320" spans="1:31" ht="43.5">
       <c r="A320" s="3" t="s">
         <v>148</v>
       </c>
@@ -31559,7 +31691,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="425" spans="1:32" ht="72.5">
+    <row r="425" spans="1:32" ht="87">
       <c r="A425" s="3" t="s">
         <v>194</v>
       </c>
@@ -36642,6 +36774,12 @@
       <c r="E597">
         <f>COUNTA(A1:A594)</f>
         <v>594</v>
+      </c>
+    </row>
+    <row r="600" spans="1:22">
+      <c r="E600">
+        <f>COUNTIF(F:F, "Autograph transcript error, but still a variant") + COUNTIF(F:F, "Apograph transcript error, but still a variant") + COUNTIF(F:F, "Not a variant: autograph transcript error") + COUNTIF(F:F, "Not a variant: apograph transcript error")</f>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -36801,37 +36939,37 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{544BCAA1-F71E-41AE-9339-D560C6EF2BFC}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
+            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Y2:Y1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{86558D7A-0079-4183-BEBD-EAC07C0B3396}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
+            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Z2:Z1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1E18B083-969A-4C72-8333-825D16438F2D}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
+            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AA2:AA1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CCE3C97A-CC8E-4E7A-83D1-60C59A5C6F5E}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
+            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AB2:AB1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4BFBF9CE-E7E2-4E15-BB49-97EF2D8683FC}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
+            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AD2:AD1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8FB8C1AC-F008-4C8D-80B6-1E37F0F2E67D}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
+            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AE2:AE1048576</xm:sqref>
         </x14:dataValidation>
@@ -36843,13 +36981,13 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{ADA4A2FA-8AE6-4C83-BF91-235140C72886}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$I$2:$I$1048576</xm:f>
+            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X1048576</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{551ECDE9-28E9-43BB-9EFF-3B7CC6890FCF}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+            <xm:f>'Data Regularization'!$Q$2:$Q$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AF2:AF1048576</xm:sqref>
         </x14:dataValidation>
@@ -37029,10 +37167,10 @@
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C933DA8F-F5EE-4CC3-9266-3537A650885B}">
-  <dimension ref="A1:P21"/>
+  <dimension ref="A1:Q21"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:16">
+    <row r="1" spans="1:17">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -37058,34 +37196,37 @@
         <v>1384</v>
       </c>
       <c r="I1" s="1" t="s">
+        <v>1645</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>1385</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>1386</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>1340</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>1341</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>1342</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>1387</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>1343</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>1388</v>
       </c>
     </row>
-    <row r="2" spans="1:16">
+    <row r="2" spans="1:17">
       <c r="A2" s="1"/>
     </row>
-    <row r="3" spans="1:16">
+    <row r="3" spans="1:17">
       <c r="A3" t="s">
         <v>554</v>
       </c>
@@ -37111,31 +37252,34 @@
         <v>4</v>
       </c>
       <c r="I3" t="s">
+        <v>1646</v>
+      </c>
+      <c r="J3" t="s">
         <v>557</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>4</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>1347</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>557</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>1348</v>
       </c>
-      <c r="N3" t="s">
+      <c r="O3" t="s">
         <v>557</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>1349</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>557</v>
       </c>
     </row>
-    <row r="4" spans="1:16">
+    <row r="4" spans="1:17">
       <c r="A4" t="s">
         <v>559</v>
       </c>
@@ -37161,31 +37305,34 @@
         <v>1389</v>
       </c>
       <c r="I4" t="s">
+        <v>1647</v>
+      </c>
+      <c r="J4" t="s">
         <v>564</v>
       </c>
-      <c r="J4" t="s">
+      <c r="K4" t="s">
         <v>1389</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>1566</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>564</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>1354</v>
       </c>
-      <c r="N4" t="s">
+      <c r="O4" t="s">
         <v>564</v>
       </c>
-      <c r="O4" t="s">
+      <c r="P4" t="s">
         <v>1355</v>
       </c>
-      <c r="P4" t="s">
+      <c r="Q4" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="5" spans="1:16">
+    <row r="5" spans="1:17">
       <c r="A5" t="s">
         <v>563</v>
       </c>
@@ -37204,17 +37351,20 @@
       <c r="F5" t="s">
         <v>1391</v>
       </c>
-      <c r="K5" t="s">
+      <c r="I5" t="s">
+        <v>1609</v>
+      </c>
+      <c r="L5" t="s">
         <v>1353</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>1357</v>
       </c>
-      <c r="O5" t="s">
+      <c r="P5" t="s">
         <v>1358</v>
       </c>
     </row>
-    <row r="6" spans="1:16">
+    <row r="6" spans="1:17">
       <c r="A6" t="s">
         <v>566</v>
       </c>
@@ -37227,14 +37377,14 @@
       <c r="E6" t="s">
         <v>1359</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>1360</v>
       </c>
-      <c r="O6" t="s">
+      <c r="P6" t="s">
         <v>1361</v>
       </c>
     </row>
-    <row r="7" spans="1:16">
+    <row r="7" spans="1:17">
       <c r="A7" t="s">
         <v>576</v>
       </c>
@@ -37244,11 +37394,11 @@
       <c r="E7" t="s">
         <v>1362</v>
       </c>
-      <c r="M7" t="s">
+      <c r="N7" t="s">
         <v>1396</v>
       </c>
     </row>
-    <row r="8" spans="1:16">
+    <row r="8" spans="1:17">
       <c r="A8" t="s">
         <v>577</v>
       </c>
@@ -37258,11 +37408,11 @@
       <c r="E8" t="s">
         <v>1364</v>
       </c>
-      <c r="M8" t="s">
+      <c r="N8" t="s">
         <v>1363</v>
       </c>
     </row>
-    <row r="9" spans="1:16">
+    <row r="9" spans="1:17">
       <c r="A9" t="s">
         <v>10</v>
       </c>
@@ -37272,11 +37422,11 @@
       <c r="E9" t="s">
         <v>1366</v>
       </c>
-      <c r="M9" t="s">
+      <c r="N9" t="s">
         <v>1365</v>
       </c>
     </row>
-    <row r="10" spans="1:16">
+    <row r="10" spans="1:17">
       <c r="A10" t="s">
         <v>568</v>
       </c>
@@ -37286,44 +37436,44 @@
       <c r="E10" t="s">
         <v>1368</v>
       </c>
-      <c r="M10" t="s">
+      <c r="N10" t="s">
         <v>1367</v>
       </c>
     </row>
-    <row r="11" spans="1:16">
+    <row r="11" spans="1:17">
       <c r="A11" t="s">
         <v>555</v>
       </c>
       <c r="E11" t="s">
         <v>1370</v>
       </c>
-      <c r="M11" t="s">
+      <c r="N11" t="s">
         <v>1369</v>
       </c>
     </row>
-    <row r="12" spans="1:16">
+    <row r="12" spans="1:17">
       <c r="A12" t="s">
         <v>1394</v>
       </c>
       <c r="E12" t="s">
         <v>1395</v>
       </c>
-      <c r="M12" t="s">
+      <c r="N12" t="s">
         <v>1494</v>
       </c>
     </row>
-    <row r="13" spans="1:16">
+    <row r="13" spans="1:17">
       <c r="A13" t="s">
         <v>574</v>
       </c>
       <c r="E13" t="s">
         <v>1397</v>
       </c>
-      <c r="M13" t="s">
+      <c r="N13" t="s">
         <v>1495</v>
       </c>
     </row>
-    <row r="14" spans="1:16">
+    <row r="14" spans="1:17">
       <c r="A14" t="s">
         <v>575</v>
       </c>
@@ -37331,12 +37481,12 @@
         <v>1371</v>
       </c>
     </row>
-    <row r="15" spans="1:16">
+    <row r="15" spans="1:17">
       <c r="A15" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="16" spans="1:16">
+    <row r="16" spans="1:17">
       <c r="A16" t="s">
         <v>556</v>
       </c>
@@ -37379,7 +37529,7 @@
   <cols>
     <col min="1" max="1" width="11.453125" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="20.81640625" customWidth="1"/>
-    <col min="4" max="6" width="8.7265625" hidden="1" customWidth="1"/>
+    <col min="4" max="6" width="8.7265625" customWidth="1"/>
     <col min="11" max="29" width="8.90625" customWidth="1"/>
   </cols>
   <sheetData>
@@ -43444,37 +43594,37 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4007FB69-E1E6-4C3A-A828-89392DBD3885}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
+            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>V2:V124</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A45F9981-851C-4449-B1D8-8BC63CB6B375}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
+            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>W2:W124</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B999C6F3-9800-46C7-AC94-CCCA1D72DE93}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
+            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X124</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{178A33A0-792A-4D5A-9496-018F388C615E}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
+            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Y2:Y124</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C401B9F8-33E9-4821-B836-28EC14A98128}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
+            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AA2:AA124</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C780CE18-7DD0-4EDE-B8A5-D11BBE966671}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
+            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AB2:AB124</xm:sqref>
         </x14:dataValidation>
@@ -43486,13 +43636,13 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{2A377462-BC6B-487A-A7DF-63EBC1F044A9}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$I$2:$I$1048576</xm:f>
+            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>U2:U124</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{18E3B7E9-4F1C-452A-97D7-81675A173845}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+            <xm:f>'Data Regularization'!$Q$2:$Q$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AC2:AC124</xm:sqref>
         </x14:dataValidation>
@@ -43504,6 +43654,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{84A221FA-E89D-461A-AA52-BC719CEBB42E}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:AG100"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <cols>
@@ -43605,7 +43756,7 @@
         <v>1572</v>
       </c>
     </row>
-    <row r="2" spans="1:31" ht="58">
+    <row r="2" spans="1:31" ht="58" hidden="1">
       <c r="A2" s="3" t="s">
         <v>15</v>
       </c>
@@ -43779,7 +43930,7 @@
       <c r="AC4" s="7"/>
       <c r="AD4" s="7"/>
     </row>
-    <row r="5" spans="1:31" ht="275.5">
+    <row r="5" spans="1:31" ht="290" hidden="1">
       <c r="A5" s="3" t="s">
         <v>27</v>
       </c>
@@ -43835,7 +43986,7 @@
       <c r="AC5" s="7"/>
       <c r="AD5" s="7"/>
     </row>
-    <row r="6" spans="1:31" ht="261">
+    <row r="6" spans="1:31" ht="290" hidden="1">
       <c r="A6" s="3" t="s">
         <v>27</v>
       </c>
@@ -43894,7 +44045,7 @@
       <c r="AC6" s="7"/>
       <c r="AD6" s="7"/>
     </row>
-    <row r="7" spans="1:31" ht="87">
+    <row r="7" spans="1:31" ht="101.5" hidden="1">
       <c r="A7" s="3" t="s">
         <v>35</v>
       </c>
@@ -44056,7 +44207,7 @@
       <c r="AC9" s="7"/>
       <c r="AD9" s="7"/>
     </row>
-    <row r="10" spans="1:31" ht="58">
+    <row r="10" spans="1:31" ht="58" hidden="1">
       <c r="A10" s="3" t="s">
         <v>42</v>
       </c>
@@ -44168,7 +44319,7 @@
       <c r="AC11" s="7"/>
       <c r="AD11" s="7"/>
     </row>
-    <row r="12" spans="1:31" ht="87">
+    <row r="12" spans="1:31" ht="87" hidden="1">
       <c r="A12" s="3" t="s">
         <v>64</v>
       </c>
@@ -44281,7 +44432,7 @@
       <c r="AC13" s="7"/>
       <c r="AD13" s="7"/>
     </row>
-    <row r="14" spans="1:31" ht="29">
+    <row r="14" spans="1:31" ht="29" hidden="1">
       <c r="A14" s="3" t="s">
         <v>74</v>
       </c>
@@ -44447,7 +44598,7 @@
       <c r="AC16" s="7"/>
       <c r="AD16" s="7"/>
     </row>
-    <row r="17" spans="1:30" ht="29">
+    <row r="17" spans="1:30" ht="29" hidden="1">
       <c r="A17" s="3" t="s">
         <v>93</v>
       </c>
@@ -44555,7 +44706,7 @@
       <c r="AC18" s="7"/>
       <c r="AD18" s="7"/>
     </row>
-    <row r="19" spans="1:30" ht="116">
+    <row r="19" spans="1:30" ht="130.5">
       <c r="A19" s="3" t="s">
         <v>109</v>
       </c>
@@ -44607,7 +44758,7 @@
       <c r="AC19" s="7"/>
       <c r="AD19" s="7"/>
     </row>
-    <row r="20" spans="1:30" ht="43.5">
+    <row r="20" spans="1:30" ht="43.5" hidden="1">
       <c r="A20" s="3" t="s">
         <v>114</v>
       </c>
@@ -44718,7 +44869,7 @@
       <c r="AC21" s="7"/>
       <c r="AD21" s="7"/>
     </row>
-    <row r="22" spans="1:30" ht="58">
+    <row r="22" spans="1:30" ht="58" hidden="1">
       <c r="A22" s="3" t="s">
         <v>133</v>
       </c>
@@ -44772,7 +44923,7 @@
       <c r="AC22" s="7"/>
       <c r="AD22" s="7"/>
     </row>
-    <row r="23" spans="1:30" ht="43.5">
+    <row r="23" spans="1:30" ht="58">
       <c r="A23" s="3" t="s">
         <v>141</v>
       </c>
@@ -44936,7 +45087,7 @@
       <c r="AC25" s="7"/>
       <c r="AD25" s="7"/>
     </row>
-    <row r="26" spans="1:30" ht="87">
+    <row r="26" spans="1:30" ht="87" hidden="1">
       <c r="A26" s="3" t="s">
         <v>148</v>
       </c>
@@ -44994,7 +45145,7 @@
       <c r="AC26" s="7"/>
       <c r="AD26" s="7"/>
     </row>
-    <row r="27" spans="1:30" ht="43.5">
+    <row r="27" spans="1:30" ht="43.5" hidden="1">
       <c r="A27" s="3" t="s">
         <v>150</v>
       </c>
@@ -45055,7 +45206,7 @@
       <c r="AC27" s="7"/>
       <c r="AD27" s="7"/>
     </row>
-    <row r="28" spans="1:30" ht="29">
+    <row r="28" spans="1:30" ht="29" hidden="1">
       <c r="A28" s="3" t="s">
         <v>152</v>
       </c>
@@ -45163,7 +45314,7 @@
       <c r="AC29" s="7"/>
       <c r="AD29" s="7"/>
     </row>
-    <row r="30" spans="1:30" ht="43.5">
+    <row r="30" spans="1:30" ht="43.5" hidden="1">
       <c r="A30" s="3" t="s">
         <v>159</v>
       </c>
@@ -45221,7 +45372,7 @@
       <c r="AC30" s="7"/>
       <c r="AD30" s="7"/>
     </row>
-    <row r="31" spans="1:30" ht="43.5">
+    <row r="31" spans="1:30" ht="43.5" hidden="1">
       <c r="A31" s="3" t="s">
         <v>161</v>
       </c>
@@ -45329,7 +45480,7 @@
       <c r="AC32" s="7"/>
       <c r="AD32" s="7"/>
     </row>
-    <row r="33" spans="1:33" ht="116">
+    <row r="33" spans="1:33" ht="116" hidden="1">
       <c r="A33" s="3" t="s">
         <v>175</v>
       </c>
@@ -45387,7 +45538,7 @@
       <c r="AC33" s="7"/>
       <c r="AD33" s="7"/>
     </row>
-    <row r="34" spans="1:33" ht="29">
+    <row r="34" spans="1:33" ht="43.5" hidden="1">
       <c r="A34" s="3" t="s">
         <v>177</v>
       </c>
@@ -45495,7 +45646,7 @@
       <c r="AC35" s="7"/>
       <c r="AD35" s="7"/>
     </row>
-    <row r="36" spans="1:33" ht="58">
+    <row r="36" spans="1:33" ht="58" hidden="1">
       <c r="A36" s="3" t="s">
         <v>192</v>
       </c>
@@ -45666,7 +45817,7 @@
       <c r="AC38" s="7"/>
       <c r="AD38" s="7"/>
     </row>
-    <row r="39" spans="1:33" ht="29">
+    <row r="39" spans="1:33" ht="29" hidden="1">
       <c r="A39" s="3" t="s">
         <v>210</v>
       </c>
@@ -45720,7 +45871,7 @@
       <c r="AC39" s="7"/>
       <c r="AD39" s="7"/>
     </row>
-    <row r="40" spans="1:33" ht="43.5">
+    <row r="40" spans="1:33" ht="43.5" hidden="1">
       <c r="A40" s="3" t="s">
         <v>215</v>
       </c>
@@ -45774,7 +45925,7 @@
       <c r="AC40" s="7"/>
       <c r="AD40" s="7"/>
     </row>
-    <row r="41" spans="1:33" ht="43.5">
+    <row r="41" spans="1:33" ht="58" hidden="1">
       <c r="A41" s="3" t="s">
         <v>228</v>
       </c>
@@ -45841,7 +45992,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="42" spans="1:33" ht="87">
+    <row r="42" spans="1:33" ht="101.5" hidden="1">
       <c r="A42" s="3" t="s">
         <v>228</v>
       </c>
@@ -45971,7 +46122,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="44" spans="1:33" ht="72.5">
+    <row r="44" spans="1:33" ht="72.5" hidden="1">
       <c r="A44" s="3" t="s">
         <v>231</v>
       </c>
@@ -46034,7 +46185,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="45" spans="1:33" ht="72.5">
+    <row r="45" spans="1:33" ht="72.5" hidden="1">
       <c r="A45" s="3" t="s">
         <v>237</v>
       </c>
@@ -46099,7 +46250,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="46" spans="1:33" ht="58">
+    <row r="46" spans="1:33" ht="58" hidden="1">
       <c r="A46" s="3" t="s">
         <v>241</v>
       </c>
@@ -46162,7 +46313,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="47" spans="1:33" ht="43.5">
+    <row r="47" spans="1:33" ht="58" hidden="1">
       <c r="A47" s="3" t="s">
         <v>249</v>
       </c>
@@ -46225,7 +46376,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="48" spans="1:33" ht="116">
+    <row r="48" spans="1:33" ht="116" hidden="1">
       <c r="A48" s="3" t="s">
         <v>254</v>
       </c>
@@ -46774,6 +46925,13 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:AG48" xr:uid="{84A221FA-E89D-461A-AA52-BC719CEBB42E}">
+    <filterColumn colId="6">
+      <filters>
+        <filter val="Omission"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <mergeCells count="1">
     <mergeCell ref="D67:F67"/>
   </mergeCells>
@@ -46953,37 +47111,37 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C0620754-77B3-44B0-8430-51B0224827B6}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
+            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>W2:W48</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{926302F9-21DC-4EC1-9E0D-2BB135A6A786}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
+            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X48</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1C6EE915-AE23-42C6-A86C-447865784B4C}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
+            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Y2:Y48</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7E31E6D6-B288-4D4B-BDD9-7048D13B96BD}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
+            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Z2:Z48</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{37B508C1-16E4-4C32-BAD0-AD322590C77C}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
+            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AB2:AB48</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{C18E595F-332C-4631-805B-2956A14A1C3A}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
+            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AC2:AC48</xm:sqref>
         </x14:dataValidation>
@@ -46995,13 +47153,13 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{158CAB09-7C18-4BFA-9588-AA746FE031CC}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$I$2:$I$1048576</xm:f>
+            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>V2:V48</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{672AB143-E130-4ABB-8873-FA7D999CCFA7}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+            <xm:f>'Data Regularization'!$Q$2:$Q$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AD2:AD48</xm:sqref>
         </x14:dataValidation>
@@ -47166,7 +47324,7 @@
       <c r="AC2" s="7"/>
       <c r="AD2" s="7"/>
     </row>
-    <row r="3" spans="1:31" ht="87">
+    <row r="3" spans="1:31" ht="101.5">
       <c r="A3" s="3" t="s">
         <v>35</v>
       </c>
@@ -48248,7 +48406,7 @@
       <c r="AC22" s="7"/>
       <c r="AD22" s="7"/>
     </row>
-    <row r="23" spans="1:33" ht="29">
+    <row r="23" spans="1:33" ht="43.5">
       <c r="A23" s="3" t="s">
         <v>177</v>
       </c>
@@ -48705,7 +48863,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="31" spans="1:33" ht="43.5">
+    <row r="31" spans="1:33" ht="58">
       <c r="A31" s="3" t="s">
         <v>249</v>
       </c>
@@ -49061,13 +49219,13 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="16">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4FF62DCB-3CDD-480D-A927-C465D4F5DB09}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+            <xm:f>'Data Regularization'!$Q$2:$Q$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AD2:AD32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{8041A7FA-B96B-4D91-8778-D6963171AD6D}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$I$2:$I$1048576</xm:f>
+            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>V2:V32</xm:sqref>
         </x14:dataValidation>
@@ -49079,37 +49237,37 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4C41C204-8356-485B-9D32-0B83B49A75C3}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
+            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AC2:AC32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{F595DA8D-F31B-45EA-8392-33A2022A0925}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
+            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AB2:AB32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{50B84040-ABC0-464F-92EF-4AD98F2A3BF8}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
+            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Z2:Z32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{9C55F5F9-998E-4245-862C-7351B9600608}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
+            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Y2:Y32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{D832FC60-DA0E-4C8D-9D26-F51C1942D779}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
+            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X32</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FCCA2196-20F7-4E4F-8C7F-E0FAC50E43E0}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
+            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>W2:W32</xm:sqref>
         </x14:dataValidation>
@@ -49541,7 +49699,7 @@
       <c r="AC6" s="7"/>
       <c r="AD6" s="7"/>
     </row>
-    <row r="7" spans="1:33" ht="43.5">
+    <row r="7" spans="1:33" ht="58">
       <c r="A7" s="3" t="s">
         <v>228</v>
       </c>
@@ -49607,7 +49765,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="8" spans="1:33" ht="87">
+    <row r="8" spans="1:33" ht="101.5">
       <c r="A8" s="3" t="s">
         <v>228</v>
       </c>
@@ -49876,13 +50034,13 @@
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="16">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E383AFF4-A52F-430A-8DC5-A0B499A4DE73}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+            <xm:f>'Data Regularization'!$Q$2:$Q$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AD2:AD8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{7771EBFA-97E7-4C99-88A9-6080EC3BF779}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$I$2:$I$1048576</xm:f>
+            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>V2:V8</xm:sqref>
         </x14:dataValidation>
@@ -49894,37 +50052,37 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CEB9EC37-E552-4937-9272-CC35E28DB432}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
+            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AC2:AC8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{3F268A4B-4C94-4922-B837-41359B6E91F8}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
+            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AB2:AB8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FFCF9CDD-07DD-4EDC-81DA-9B869D274C6E}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
+            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Z2:Z8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{BCEBA13C-8E06-415A-806C-5DC79A4017D0}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
+            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Y2:Y8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{90F12384-00C8-49C3-A5B7-E4B083774396}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
+            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X8</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{4F0C9E83-1779-4235-9711-867F86331CDC}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
+            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>W2:W8</xm:sqref>
         </x14:dataValidation>
@@ -50730,7 +50888,7 @@
       <c r="AE13" s="7"/>
       <c r="AF13" s="7"/>
     </row>
-    <row r="14" spans="1:32" ht="116">
+    <row r="14" spans="1:32" ht="130.5">
       <c r="A14" s="3" t="s">
         <v>109</v>
       </c>
@@ -51785,37 +51943,37 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E7C52A28-4741-4A9A-A78A-8588C0AE851C}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
+            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Y2:Y27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{94BFA744-D38C-4369-8FC2-1DE507B62DDF}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
+            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Z2:Z27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7D8BCE44-873C-406C-B50A-630126E88264}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
+            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AA2:AA27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{A741226C-E3D8-4541-9D92-C8D375E9B5DB}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
+            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AB2:AB27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{7AEB8B38-FBF9-4EA5-B70F-7D2A50BFA712}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
+            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AD2:AD27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1DCAA841-27AE-4E00-A8F4-A3B04E2D5B80}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
+            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AE2:AE27</xm:sqref>
         </x14:dataValidation>
@@ -51827,13 +51985,13 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{6282FD0B-0D54-42B6-ABBF-E2774E1C2DEC}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$I$2:$I$1048576</xm:f>
+            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X27</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{70D13D62-D971-4C7A-9655-567551BC1323}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+            <xm:f>'Data Regularization'!$Q$2:$Q$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AF2:AF27</xm:sqref>
         </x14:dataValidation>
@@ -51845,10 +52003,10 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79471631-29FB-4EB4-AAE7-2BB809120F9D}">
-  <dimension ref="A1:AD14"/>
+  <dimension ref="A1:AE21"/>
   <sheetFormatPr defaultRowHeight="14.5"/>
   <sheetData>
-    <row r="1" spans="1:30" s="1" customFormat="1">
+    <row r="1" spans="1:31" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -51913,34 +52071,37 @@
         <v>1384</v>
       </c>
       <c r="V1" s="1" t="s">
+        <v>1645</v>
+      </c>
+      <c r="W1" s="1" t="s">
         <v>1385</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="X1" s="1" t="s">
         <v>1386</v>
       </c>
-      <c r="X1" s="1" t="s">
+      <c r="Y1" s="1" t="s">
         <v>1340</v>
       </c>
-      <c r="Y1" s="1" t="s">
+      <c r="Z1" s="1" t="s">
         <v>1341</v>
       </c>
-      <c r="Z1" s="1" t="s">
+      <c r="AA1" s="1" t="s">
         <v>1342</v>
       </c>
-      <c r="AA1" s="1" t="s">
+      <c r="AB1" s="1" t="s">
         <v>1383</v>
       </c>
-      <c r="AB1" s="1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>1387</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>1343</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>1388</v>
       </c>
     </row>
-    <row r="2" spans="1:30" ht="130.5">
+    <row r="2" spans="1:31" ht="130.5">
       <c r="A2" s="3" t="s">
         <v>16</v>
       </c>
@@ -51990,7 +52151,9 @@
       <c r="U2" s="7" t="s">
         <v>1389</v>
       </c>
-      <c r="V2" s="7"/>
+      <c r="V2" s="7" t="s">
+        <v>1646</v>
+      </c>
       <c r="W2" s="7"/>
       <c r="X2" s="7"/>
       <c r="Y2" s="7"/>
@@ -51999,8 +52162,9 @@
       <c r="AB2" s="7"/>
       <c r="AC2" s="7"/>
       <c r="AD2" s="7"/>
-    </row>
-    <row r="3" spans="1:30" ht="101.5">
+      <c r="AE2" s="7"/>
+    </row>
+    <row r="3" spans="1:31" ht="101.5">
       <c r="A3" s="3" t="s">
         <v>19</v>
       </c>
@@ -52045,7 +52209,9 @@
       <c r="U3" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="V3" s="7"/>
+      <c r="V3" s="7" t="s">
+        <v>1609</v>
+      </c>
       <c r="W3" s="7"/>
       <c r="X3" s="7"/>
       <c r="Y3" s="7"/>
@@ -52054,8 +52220,9 @@
       <c r="AB3" s="7"/>
       <c r="AC3" s="7"/>
       <c r="AD3" s="7"/>
-    </row>
-    <row r="4" spans="1:30" ht="43.5">
+      <c r="AE3" s="7"/>
+    </row>
+    <row r="4" spans="1:31" ht="43.5">
       <c r="A4" s="3" t="s">
         <v>142</v>
       </c>
@@ -52090,7 +52257,9 @@
       <c r="U4" s="7" t="s">
         <v>1389</v>
       </c>
-      <c r="V4" s="7"/>
+      <c r="V4" s="7" t="s">
+        <v>1647</v>
+      </c>
       <c r="W4" s="7"/>
       <c r="X4" s="7"/>
       <c r="Y4" s="7"/>
@@ -52099,8 +52268,9 @@
       <c r="AB4" s="7"/>
       <c r="AC4" s="7"/>
       <c r="AD4" s="7"/>
-    </row>
-    <row r="5" spans="1:30" ht="43.5">
+      <c r="AE4" s="7"/>
+    </row>
+    <row r="5" spans="1:31" ht="43.5">
       <c r="A5" s="3" t="s">
         <v>143</v>
       </c>
@@ -52135,7 +52305,9 @@
       <c r="U5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="V5" s="7"/>
+      <c r="V5" s="7" t="s">
+        <v>1646</v>
+      </c>
       <c r="W5" s="7"/>
       <c r="X5" s="7"/>
       <c r="Y5" s="7"/>
@@ -52144,8 +52316,9 @@
       <c r="AB5" s="7"/>
       <c r="AC5" s="7"/>
       <c r="AD5" s="7"/>
-    </row>
-    <row r="6" spans="1:30" ht="43.5">
+      <c r="AE5" s="7"/>
+    </row>
+    <row r="6" spans="1:31" ht="43.5">
       <c r="A6" s="3" t="s">
         <v>143</v>
       </c>
@@ -52190,7 +52363,9 @@
       <c r="U6" s="7" t="s">
         <v>1389</v>
       </c>
-      <c r="V6" s="7"/>
+      <c r="V6" s="7" t="s">
+        <v>1646</v>
+      </c>
       <c r="W6" s="7"/>
       <c r="X6" s="7"/>
       <c r="Y6" s="7"/>
@@ -52199,8 +52374,9 @@
       <c r="AB6" s="7"/>
       <c r="AC6" s="7"/>
       <c r="AD6" s="7"/>
-    </row>
-    <row r="7" spans="1:30" ht="29">
+      <c r="AE6" s="7"/>
+    </row>
+    <row r="7" spans="1:31" ht="29">
       <c r="A7" s="3" t="s">
         <v>145</v>
       </c>
@@ -52245,7 +52421,9 @@
       <c r="U7" s="7" t="s">
         <v>1389</v>
       </c>
-      <c r="V7" s="7"/>
+      <c r="V7" s="7" t="s">
+        <v>1646</v>
+      </c>
       <c r="W7" s="7"/>
       <c r="X7" s="7"/>
       <c r="Y7" s="7"/>
@@ -52254,8 +52432,9 @@
       <c r="AB7" s="7"/>
       <c r="AC7" s="7"/>
       <c r="AD7" s="7"/>
-    </row>
-    <row r="8" spans="1:30">
+      <c r="AE7" s="7"/>
+    </row>
+    <row r="8" spans="1:31">
       <c r="A8" s="3" t="s">
         <v>193</v>
       </c>
@@ -52290,7 +52469,9 @@
       <c r="U8" s="7" t="s">
         <v>1389</v>
       </c>
-      <c r="V8" s="7"/>
+      <c r="V8" s="7" t="s">
+        <v>1647</v>
+      </c>
       <c r="W8" s="7"/>
       <c r="X8" s="7"/>
       <c r="Y8" s="7"/>
@@ -52299,8 +52480,9 @@
       <c r="AB8" s="7"/>
       <c r="AC8" s="7"/>
       <c r="AD8" s="7"/>
-    </row>
-    <row r="9" spans="1:30" ht="232">
+      <c r="AE8" s="7"/>
+    </row>
+    <row r="9" spans="1:31" ht="232">
       <c r="A9" s="3" t="s">
         <v>194</v>
       </c>
@@ -52335,7 +52517,9 @@
       <c r="U9" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="V9" s="7"/>
+      <c r="V9" s="7" t="s">
+        <v>1647</v>
+      </c>
       <c r="W9" s="7"/>
       <c r="X9" s="7"/>
       <c r="Y9" s="7"/>
@@ -52344,8 +52528,9 @@
       <c r="AB9" s="7"/>
       <c r="AC9" s="7"/>
       <c r="AD9" s="7"/>
-    </row>
-    <row r="12" spans="1:30">
+      <c r="AE9" s="7"/>
+    </row>
+    <row r="12" spans="1:31">
       <c r="D12" t="s">
         <v>1558</v>
       </c>
@@ -52354,7 +52539,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:30">
+    <row r="13" spans="1:31">
       <c r="D13" t="s">
         <v>1559</v>
       </c>
@@ -52363,7 +52548,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:30">
+    <row r="14" spans="1:31">
       <c r="D14" t="s">
         <v>1560</v>
       </c>
@@ -52372,7 +52557,125 @@
         <v>0.375</v>
       </c>
     </row>
+    <row r="17" spans="4:10">
+      <c r="E17" s="13" t="s">
+        <v>1648</v>
+      </c>
+      <c r="F17" s="13"/>
+      <c r="G17" s="13"/>
+      <c r="H17" s="13"/>
+    </row>
+    <row r="18" spans="4:10">
+      <c r="E18" t="s">
+        <v>1649</v>
+      </c>
+      <c r="F18" t="s">
+        <v>1650</v>
+      </c>
+      <c r="G18" t="s">
+        <v>1651</v>
+      </c>
+      <c r="H18" t="s">
+        <v>1652</v>
+      </c>
+      <c r="I18" t="s">
+        <v>1609</v>
+      </c>
+      <c r="J18" t="s">
+        <v>1517</v>
+      </c>
+    </row>
+    <row r="19" spans="4:10">
+      <c r="D19" t="s">
+        <v>1558</v>
+      </c>
+      <c r="E19">
+        <f>COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"forward")</f>
+        <v>1</v>
+      </c>
+      <c r="F19">
+        <f>COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"forward") + COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"both")</f>
+        <v>2</v>
+      </c>
+      <c r="G19">
+        <f>COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"backward")</f>
+        <v>1</v>
+      </c>
+      <c r="H19">
+        <f>COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"backward") + COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"both")</f>
+        <v>2</v>
+      </c>
+      <c r="I19">
+        <f>COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"both")</f>
+        <v>1</v>
+      </c>
+      <c r="J19">
+        <f>COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"both") + COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"forward") + COUNTIFS($U$2:$U$9,"Harmonizing",$V$2:$V$9,"backward")</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="20" spans="4:10">
+      <c r="D20" t="s">
+        <v>1559</v>
+      </c>
+      <c r="E20">
+        <f>COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"forward")</f>
+        <v>3</v>
+      </c>
+      <c r="F20">
+        <f>COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"forward") + COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"both")</f>
+        <v>3</v>
+      </c>
+      <c r="G20">
+        <f>COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"backward")</f>
+        <v>2</v>
+      </c>
+      <c r="H20">
+        <f>COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"backward") + COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"both")</f>
+        <v>2</v>
+      </c>
+      <c r="I20">
+        <f>COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"both")</f>
+        <v>0</v>
+      </c>
+      <c r="J20">
+        <f>COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"both") + COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"forward") + COUNTIFS($U$2:$U$9,"Disharmonizing",$V$2:$V$9,"backward")</f>
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21" spans="4:10">
+      <c r="D21" t="s">
+        <v>1560</v>
+      </c>
+      <c r="E21">
+        <f t="shared" ref="E21:G21" si="0">E19/(E19+E20)</f>
+        <v>0.25</v>
+      </c>
+      <c r="F21">
+        <f t="shared" si="0"/>
+        <v>0.4</v>
+      </c>
+      <c r="G21">
+        <f t="shared" si="0"/>
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="H21">
+        <f t="shared" ref="H21:J21" si="1">H19/(H19+H20)</f>
+        <v>0.5</v>
+      </c>
+      <c r="I21">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="J21">
+        <f t="shared" si="1"/>
+        <v>0.375</v>
+      </c>
+    </row>
   </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="E17:H17"/>
+  </mergeCells>
   <conditionalFormatting sqref="H2:H9">
     <cfRule type="expression" dxfId="25" priority="4">
       <formula>$J2&lt;&gt;""</formula>
@@ -52440,18 +52743,18 @@
       <formula>"&lt;&gt;AND(LEFT($J2,3)=""Sub"", RIGHT($J2,4)&lt;&gt;""Form"")"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U9">
+  <conditionalFormatting sqref="U2:V9">
     <cfRule type="expression" dxfId="8" priority="7">
-      <formula>AND($W2&lt;&gt;"",OR($AD2="Yes",$AE2&lt;&gt;""))</formula>
+      <formula>AND($X2&lt;&gt;"",OR($AE2="Yes",$AF2&lt;&gt;""))</formula>
     </cfRule>
     <cfRule type="expression" dxfId="7" priority="8">
-      <formula>OR($AD2="Yes",$AE2&lt;&gt;"")</formula>
+      <formula>OR($AE2="Yes",$AF2&lt;&gt;"")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="6" priority="26">
-      <formula>AND($AD2&lt;&gt;"Yes",$AE2="")</formula>
+      <formula>AND($AE2&lt;&gt;"Yes",$AF2="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="U2:AD9">
+  <conditionalFormatting sqref="U2:AE9">
     <cfRule type="expression" dxfId="5" priority="24">
       <formula>AND($J2&lt;&gt;"",$J2&lt;&gt;"Unclear due to correction")</formula>
     </cfRule>
@@ -52459,22 +52762,22 @@
       <formula>OR($J2="",$J2="Unclear due to correction")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V9">
+  <conditionalFormatting sqref="W2:W9">
     <cfRule type="expression" dxfId="3" priority="6">
-      <formula>AND($J2&lt;&gt;"",$J2&lt;&gt;"Unclear due to correction",$X2="")</formula>
+      <formula>AND($J2&lt;&gt;"",$J2&lt;&gt;"Unclear due to correction",$Y2="")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="W2:W9">
+  <conditionalFormatting sqref="X2:X9">
     <cfRule type="expression" dxfId="2" priority="9">
-      <formula>AND($X2="Yes",$Y2="")</formula>
+      <formula>AND($Y2="Yes",$Z2="")</formula>
     </cfRule>
     <cfRule type="expression" dxfId="1" priority="10">
-      <formula>$X2=""</formula>
+      <formula>$Y2=""</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="AB2:AB9">
+  <conditionalFormatting sqref="AC2:AC9">
     <cfRule type="expression" dxfId="0" priority="11">
-      <formula>AND(OR($AB2&lt;&gt;"",$AC2&lt;&gt;""),$AD2="")</formula>
+      <formula>AND(OR($AC2&lt;&gt;"",$AD2&lt;&gt;""),$AE2="")</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -52482,7 +52785,7 @@
   <legacyDrawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="16">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="17">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{8832CD38-B7F2-4F6A-A717-B3A94B7FA9AE}">
           <x14:formula1>
             <xm:f>'Data Regularization'!$A$2:$A$1048576</xm:f>
@@ -52527,39 +52830,39 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{8538CE67-7120-46B7-9C49-ECAEB93B9EC7}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
-          </x14:formula1>
-          <xm:sqref>W2:W9</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B935CB47-48A5-48FC-9BF1-664F02780569}">
-          <x14:formula1>
             <xm:f>'Data Regularization'!$K$2:$K$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>X2:X9</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{16DE1680-AE1D-4EE5-A491-E363E7CD129C}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B935CB47-48A5-48FC-9BF1-664F02780569}">
           <x14:formula1>
             <xm:f>'Data Regularization'!$L$2:$L$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Y2:Y9</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1E532B69-2D65-415C-8DAE-750149F0A146}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{16DE1680-AE1D-4EE5-A491-E363E7CD129C}">
           <x14:formula1>
             <xm:f>'Data Regularization'!$M$2:$M$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>Z2:Z9</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{61CF2126-3053-4E58-B947-818A6E37A05F}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{1E532B69-2D65-415C-8DAE-750149F0A146}">
           <x14:formula1>
             <xm:f>'Data Regularization'!$N$2:$N$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>AB2:AB9</xm:sqref>
+          <xm:sqref>AA2:AA9</xm:sqref>
         </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{AF061577-2D9E-4AFD-9358-F9AD858982FF}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{61CF2126-3053-4E58-B947-818A6E37A05F}">
           <x14:formula1>
             <xm:f>'Data Regularization'!$O$2:$O$1048576</xm:f>
           </x14:formula1>
           <xm:sqref>AC2:AC9</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{AF061577-2D9E-4AFD-9358-F9AD858982FF}">
+          <x14:formula1>
+            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+          </x14:formula1>
+          <xm:sqref>AD2:AD9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{FB5B8547-3A4C-44E5-AB02-5575EFBE3149}">
           <x14:formula1>
@@ -52569,15 +52872,21 @@
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" xr:uid="{9566B6FA-0B83-4684-A62B-7B95560BFD1E}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$I$2:$I$1048576</xm:f>
+            <xm:f>'Data Regularization'!$J$2:$J$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>V2:V9</xm:sqref>
+          <xm:sqref>W2:W9</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B8E8DDAA-06AF-40F3-AD9F-792A87A1D7CE}">
           <x14:formula1>
-            <xm:f>'Data Regularization'!$P$2:$P$1048576</xm:f>
+            <xm:f>'Data Regularization'!$Q$2:$Q$1048576</xm:f>
           </x14:formula1>
-          <xm:sqref>AD2:AD9</xm:sqref>
+          <xm:sqref>AE2:AE9</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B692C423-DC6F-4B4C-AC06-CB220F12FF10}">
+          <x14:formula1>
+            <xm:f>'Data Regularization'!$I$2:$I$98576</xm:f>
+          </x14:formula1>
+          <xm:sqref>V2:V9</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>